<commit_message>
Add Danish labour productivity series (Eurostat tesem160) to workbook
Adds 21 observations of nominal labour productivity per person for
Denmark, 2005-2025, indexed on EU27_2020 = 100. This is the first
genuinely economic outcome variable in the dataset: every prior
'economic effect' measure was itself an adoption measure, so the
report's central regression was adoption on adoption.

The definition entry carries the warning the index base demands - a
rise means Denmark gained on the EU average, not that Danish
productivity grew. Those are different claims and only the first is
supported by this series.

Also corrects the observation count in the verifier, which caught both
the count and the missing definition on the first run.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ax7AbUhZ1yD3sdczLm4auu
</commit_message>
<xml_diff>
--- a/ECON1596_A2_Denmark_DataWorkbook_s4040040.xlsx
+++ b/ECON1596_A2_Denmark_DataWorkbook_s4040040.xlsx
@@ -29,7 +29,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_POLICY" sheetId="20" state="visible" r:id="rId20"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_MASTER'!$A$1:$L$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'02_MASTER'!$A$1:$L$135</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -2798,7 +2798,7 @@
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>113</t>
+          <t>134</t>
         </is>
       </c>
     </row>
@@ -7483,7 +7483,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L114"/>
+  <dimension ref="A1:L135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -13298,8 +13298,1016 @@
         </is>
       </c>
     </row>
+    <row r="115">
+      <c r="A115" s="13" t="n">
+        <v>114</v>
+      </c>
+      <c r="B115" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C115" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D115" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E115" s="13" t="n">
+        <v>2005</v>
+      </c>
+      <c r="F115" s="16" t="n">
+        <v>109.2</v>
+      </c>
+      <c r="G115" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H115" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I115" s="13" t="inlineStr"/>
+      <c r="J115" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K115" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L115" s="15" t="inlineStr"/>
+    </row>
+    <row r="116">
+      <c r="A116" s="13" t="n">
+        <v>115</v>
+      </c>
+      <c r="B116" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C116" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D116" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E116" s="13" t="n">
+        <v>2006</v>
+      </c>
+      <c r="F116" s="16" t="n">
+        <v>109.3</v>
+      </c>
+      <c r="G116" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H116" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I116" s="13" t="inlineStr"/>
+      <c r="J116" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K116" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L116" s="15" t="inlineStr"/>
+    </row>
+    <row r="117">
+      <c r="A117" s="13" t="n">
+        <v>116</v>
+      </c>
+      <c r="B117" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C117" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D117" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E117" s="13" t="n">
+        <v>2007</v>
+      </c>
+      <c r="F117" s="16" t="n">
+        <v>107.1</v>
+      </c>
+      <c r="G117" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H117" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I117" s="13" t="inlineStr"/>
+      <c r="J117" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K117" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L117" s="15" t="inlineStr"/>
+    </row>
+    <row r="118">
+      <c r="A118" s="13" t="n">
+        <v>117</v>
+      </c>
+      <c r="B118" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C118" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D118" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E118" s="13" t="n">
+        <v>2008</v>
+      </c>
+      <c r="F118" s="16" t="n">
+        <v>108.5</v>
+      </c>
+      <c r="G118" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H118" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I118" s="13" t="inlineStr"/>
+      <c r="J118" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K118" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L118" s="15" t="inlineStr"/>
+    </row>
+    <row r="119">
+      <c r="A119" s="13" t="n">
+        <v>118</v>
+      </c>
+      <c r="B119" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C119" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D119" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E119" s="13" t="n">
+        <v>2009</v>
+      </c>
+      <c r="F119" s="16" t="n">
+        <v>109.9</v>
+      </c>
+      <c r="G119" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H119" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I119" s="13" t="inlineStr"/>
+      <c r="J119" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K119" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L119" s="15" t="inlineStr"/>
+    </row>
+    <row r="120">
+      <c r="A120" s="13" t="n">
+        <v>119</v>
+      </c>
+      <c r="B120" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C120" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D120" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E120" s="13" t="n">
+        <v>2010</v>
+      </c>
+      <c r="F120" s="16" t="n">
+        <v>115</v>
+      </c>
+      <c r="G120" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H120" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I120" s="13" t="inlineStr"/>
+      <c r="J120" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K120" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L120" s="15" t="inlineStr"/>
+    </row>
+    <row r="121">
+      <c r="A121" s="13" t="n">
+        <v>120</v>
+      </c>
+      <c r="B121" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C121" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D121" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E121" s="13" t="n">
+        <v>2011</v>
+      </c>
+      <c r="F121" s="16" t="n">
+        <v>113.8</v>
+      </c>
+      <c r="G121" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H121" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I121" s="13" t="inlineStr"/>
+      <c r="J121" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K121" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L121" s="15" t="inlineStr"/>
+    </row>
+    <row r="122">
+      <c r="A122" s="13" t="n">
+        <v>121</v>
+      </c>
+      <c r="B122" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C122" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D122" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E122" s="13" t="n">
+        <v>2012</v>
+      </c>
+      <c r="F122" s="16" t="n">
+        <v>113.9</v>
+      </c>
+      <c r="G122" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H122" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I122" s="13" t="inlineStr"/>
+      <c r="J122" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K122" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L122" s="15" t="inlineStr"/>
+    </row>
+    <row r="123">
+      <c r="A123" s="13" t="n">
+        <v>122</v>
+      </c>
+      <c r="B123" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C123" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D123" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E123" s="13" t="n">
+        <v>2013</v>
+      </c>
+      <c r="F123" s="16" t="n">
+        <v>115.3</v>
+      </c>
+      <c r="G123" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H123" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I123" s="13" t="inlineStr"/>
+      <c r="J123" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K123" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L123" s="15" t="inlineStr"/>
+    </row>
+    <row r="124">
+      <c r="A124" s="13" t="n">
+        <v>123</v>
+      </c>
+      <c r="B124" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C124" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D124" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E124" s="13" t="n">
+        <v>2014</v>
+      </c>
+      <c r="F124" s="16" t="n">
+        <v>115.1</v>
+      </c>
+      <c r="G124" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H124" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I124" s="13" t="inlineStr"/>
+      <c r="J124" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K124" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L124" s="15" t="inlineStr"/>
+    </row>
+    <row r="125">
+      <c r="A125" s="13" t="n">
+        <v>124</v>
+      </c>
+      <c r="B125" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C125" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D125" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E125" s="13" t="n">
+        <v>2015</v>
+      </c>
+      <c r="F125" s="16" t="n">
+        <v>113.9</v>
+      </c>
+      <c r="G125" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H125" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I125" s="13" t="inlineStr"/>
+      <c r="J125" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K125" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L125" s="15" t="inlineStr"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="13" t="n">
+        <v>125</v>
+      </c>
+      <c r="B126" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C126" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D126" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E126" s="13" t="n">
+        <v>2016</v>
+      </c>
+      <c r="F126" s="16" t="n">
+        <v>114.1</v>
+      </c>
+      <c r="G126" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H126" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I126" s="13" t="inlineStr"/>
+      <c r="J126" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K126" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L126" s="15" t="inlineStr"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="13" t="n">
+        <v>126</v>
+      </c>
+      <c r="B127" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C127" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D127" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E127" s="13" t="n">
+        <v>2017</v>
+      </c>
+      <c r="F127" s="16" t="n">
+        <v>116.3</v>
+      </c>
+      <c r="G127" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H127" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I127" s="13" t="inlineStr"/>
+      <c r="J127" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K127" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L127" s="15" t="inlineStr"/>
+    </row>
+    <row r="128">
+      <c r="A128" s="13" t="n">
+        <v>127</v>
+      </c>
+      <c r="B128" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C128" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D128" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E128" s="13" t="n">
+        <v>2018</v>
+      </c>
+      <c r="F128" s="16" t="n">
+        <v>115.3</v>
+      </c>
+      <c r="G128" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H128" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I128" s="13" t="inlineStr"/>
+      <c r="J128" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K128" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L128" s="15" t="inlineStr"/>
+    </row>
+    <row r="129">
+      <c r="A129" s="13" t="n">
+        <v>128</v>
+      </c>
+      <c r="B129" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C129" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D129" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E129" s="13" t="n">
+        <v>2019</v>
+      </c>
+      <c r="F129" s="16" t="n">
+        <v>113.2</v>
+      </c>
+      <c r="G129" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H129" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I129" s="13" t="inlineStr"/>
+      <c r="J129" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K129" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L129" s="15" t="inlineStr"/>
+    </row>
+    <row r="130">
+      <c r="A130" s="13" t="n">
+        <v>129</v>
+      </c>
+      <c r="B130" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C130" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D130" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E130" s="13" t="n">
+        <v>2020</v>
+      </c>
+      <c r="F130" s="16" t="n">
+        <v>119.6</v>
+      </c>
+      <c r="G130" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H130" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I130" s="13" t="inlineStr"/>
+      <c r="J130" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K130" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L130" s="15" t="inlineStr"/>
+    </row>
+    <row r="131">
+      <c r="A131" s="13" t="n">
+        <v>130</v>
+      </c>
+      <c r="B131" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C131" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D131" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E131" s="13" t="n">
+        <v>2021</v>
+      </c>
+      <c r="F131" s="16" t="n">
+        <v>121</v>
+      </c>
+      <c r="G131" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H131" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I131" s="13" t="inlineStr"/>
+      <c r="J131" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K131" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L131" s="15" t="inlineStr"/>
+    </row>
+    <row r="132">
+      <c r="A132" s="13" t="n">
+        <v>131</v>
+      </c>
+      <c r="B132" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C132" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D132" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E132" s="13" t="n">
+        <v>2022</v>
+      </c>
+      <c r="F132" s="16" t="n">
+        <v>120.2</v>
+      </c>
+      <c r="G132" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H132" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I132" s="13" t="inlineStr"/>
+      <c r="J132" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K132" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L132" s="15" t="inlineStr"/>
+    </row>
+    <row r="133">
+      <c r="A133" s="13" t="n">
+        <v>132</v>
+      </c>
+      <c r="B133" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C133" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D133" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E133" s="13" t="n">
+        <v>2023</v>
+      </c>
+      <c r="F133" s="16" t="n">
+        <v>113.1</v>
+      </c>
+      <c r="G133" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H133" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I133" s="13" t="inlineStr"/>
+      <c r="J133" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K133" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L133" s="15" t="inlineStr"/>
+    </row>
+    <row r="134">
+      <c r="A134" s="13" t="n">
+        <v>133</v>
+      </c>
+      <c r="B134" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C134" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D134" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E134" s="13" t="n">
+        <v>2024</v>
+      </c>
+      <c r="F134" s="16" t="n">
+        <v>116.7</v>
+      </c>
+      <c r="G134" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H134" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I134" s="13" t="inlineStr"/>
+      <c r="J134" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K134" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L134" s="15" t="inlineStr"/>
+    </row>
+    <row r="135">
+      <c r="A135" s="13" t="n">
+        <v>134</v>
+      </c>
+      <c r="B135" s="14" t="inlineStr">
+        <is>
+          <t>DK.PRD.LP.PER</t>
+        </is>
+      </c>
+      <c r="C135" s="15" t="inlineStr">
+        <is>
+          <t>Nominal labour productivity per person</t>
+        </is>
+      </c>
+      <c r="D135" s="13" t="inlineStr">
+        <is>
+          <t>DK</t>
+        </is>
+      </c>
+      <c r="E135" s="13" t="n">
+        <v>2025</v>
+      </c>
+      <c r="F135" s="16" t="n">
+        <v>116.8</v>
+      </c>
+      <c r="G135" s="13" t="inlineStr">
+        <is>
+          <t>index</t>
+        </is>
+      </c>
+      <c r="H135" s="15" t="inlineStr">
+        <is>
+          <t>EU27_2020 = 100, current prices, PPS</t>
+        </is>
+      </c>
+      <c r="I135" s="13" t="inlineStr"/>
+      <c r="J135" s="14" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="K135" s="13" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="L135" s="15" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L114"/>
+  <autoFilter ref="A1:L135"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -13310,7 +14318,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -14170,6 +15178,43 @@
         </is>
       </c>
     </row>
+    <row r="25" ht="46" customHeight="1">
+      <c r="A25" s="23" t="inlineStr">
+        <is>
+          <t>ES8</t>
+        </is>
+      </c>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>Eurostat</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>Labour productivity per person employed and hour worked (EU27_2020=100) - custom extraction, nominal labour productivity per person, Denmark, 2005-2025</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>tesem160</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>https://ec.europa.eu/eurostat/databrowser/view/tesem160/default/table?lang=en</t>
+        </is>
+      </c>
+      <c r="F25" s="15" t="inlineStr">
+        <is>
+          <t>13 September 2026</t>
+        </is>
+      </c>
+      <c r="G25" s="15" t="inlineStr">
+        <is>
+          <t>Eurostat 2026, Labour productivity per person employed and hour worked (EU27_2020=100), dataset tesem160, last updated 9 September 2026, Eurostat, accessed 13 September 2026, &lt;https://ec.europa.eu/eurostat/databrowser/view/tesem160/default/table?lang=en&gt;.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14181,7 +15226,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C31"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -14284,424 +15329,441 @@
     <row r="7" ht="44" customHeight="1">
       <c r="A7" s="25" t="inlineStr">
         <is>
-          <t>DK.FIN.BRCH</t>
+          <t>DK.PRD.LP.PER</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>Number of retail bank branches operated by Danish credit institutions.</t>
+          <t>Nominal labour productivity per person employed, indexed so that the EU27 (2020 composition) equals 100 in each year.</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>Consolidation and digitalisation both reduce this. The series alone cannot separate the two causes.</t>
+          <t>RELATIVE measure. A rise means Denmark gained ON THE EU AVERAGE; it is not a Danish growth rate and must never be read as one. Per PERSON, so it is sensitive to part-time work - the per-HOUR variant is the cleaner productivity measure. Current prices in PPS, so nominal.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="44" customHeight="1">
       <c r="A8" s="25" t="inlineStr">
         <is>
-          <t>DK.ECM.IND.BUY</t>
+          <t>DK.FIN.BRCH</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>Individuals who purchased goods or services online in the last 12 months.</t>
+          <t>Number of retail bank branches operated by Danish credit institutions.</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>DENOMINATOR BREAK at 2020: % of individuals before, % of internet users after. Never plot 2019 with later years.</t>
+          <t>Consolidation and digitalisation both reduce this. The series alone cannot separate the two causes.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="44" customHeight="1">
       <c r="A9" s="25" t="inlineStr">
         <is>
-          <t>DK.ECM.ENT.TRN</t>
+          <t>DK.ECM.IND.BUY</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>E-commerce sales as a share of total enterprise turnover.</t>
+          <t>Individuals who purchased goods or services online in the last 12 months.</t>
         </is>
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>Measures INTENSITY of online selling, not how many firms sell online. Pair with DK.ECM.ENT.SHR.</t>
+          <t>DENOMINATOR BREAK at 2020: % of individuals before, % of internet users after. Never plot 2019 with later years.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1">
       <c r="A10" s="25" t="inlineStr">
         <is>
-          <t>DK.ECM.ENT.SHR</t>
+          <t>DK.ECM.ENT.TRN</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>Share of enterprises making any e-sales.</t>
+          <t>E-commerce sales as a share of total enterprise turnover.</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>Measures BREADTH of adoption. Flat breadth with rising intensity means incumbents deepening, not new entrants.</t>
+          <t>Measures INTENSITY of online selling, not how many firms sell online. Pair with DK.ECM.ENT.SHR.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="44" customHeight="1">
       <c r="A11" s="25" t="inlineStr">
         <is>
-          <t>DK.DGP.EXMP</t>
+          <t>DK.ECM.ENT.SHR</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>Citizens formally exempt from mandatory Digital Post under the statutory exemption regime.</t>
+          <t>Share of enterprises making any e-sales.</t>
         </is>
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>An administrative status, not a measure of capability. A citizen may struggle without being exempt.</t>
+          <t>Measures BREADTH of adoption. Flat breadth with rising intensity means incumbents deepening, not new entrants.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="44" customHeight="1">
       <c r="A12" s="25" t="inlineStr">
         <is>
-          <t>DK.DGX.DIFF</t>
+          <t>DK.DGP.EXMP</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>Population estimated to face difficulties using digital public services.</t>
+          <t>Citizens formally exempt from mandatory Digital Post under the statutory exemption regime.</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>A capability estimate, not an administrative count. Much larger than the exemption rate - that gap is the analytical point.</t>
+          <t>An administrative status, not a measure of capability. A citizen may struggle without being exempt.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="44" customHeight="1">
       <c r="A13" s="25" t="inlineStr">
         <is>
-          <t>DK.DGX.JUST</t>
+          <t>DK.DGX.DIFF</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>Justitia's estimate of the digitally disadvantaged adult population.</t>
+          <t>Population estimated to face difficulties using digital public services.</t>
         </is>
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>Think-tank estimate, broadest definition of the five. Cite as an upper bound, not as an official statistic.</t>
+          <t>A capability estimate, not an administrative count. Much larger than the exemption rate - that gap is the analytical point.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="44" customHeight="1">
       <c r="A14" s="25" t="inlineStr">
         <is>
-          <t>DK.GOV.DPS.CIT</t>
+          <t>DK.DGX.JUST</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>eGovernment Benchmark composite score for citizen-facing digital public services.</t>
+          <t>Justitia's estimate of the digitally disadvantaged adult population.</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>A composite index, not a usage rate. Denmark scores BELOW the EU average despite near-universal mandated use.</t>
+          <t>Think-tank estimate, broadest definition of the five. Cite as an upper bound, not as an official statistic.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="44" customHeight="1">
       <c r="A15" s="25" t="inlineStr">
         <is>
-          <t>DK.ENV.WEEE</t>
+          <t>DK.GOV.DPS.CIT</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>Share of collected ICT-related electrical waste recycled or prepared for reuse.</t>
+          <t>eGovernment Benchmark composite score for citizen-facing digital public services.</t>
         </is>
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>Covers two WEEE categories only. Denominator is waste COLLECTED, not waste generated.</t>
+          <t>A composite index, not a usage rate. Denmark scores BELOW the EU average despite near-universal mandated use.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="44" customHeight="1">
       <c r="A16" s="25" t="inlineStr">
         <is>
-          <t>DK.PAY.DIG.POS.NUM, DK.PAY.DIG.POS.VAL</t>
+          <t>DK.ENV.WEEE</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>Digital share of physical-retail payments, by NUMBER and by VALUE respectively.</t>
+          <t>Share of collected ICT-related electrical waste recycled or prepared for reuse.</t>
         </is>
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>Two different denominators. The value share exceeds the number share because cash survives in small transactions. Never quote one as the other, and never average them.</t>
+          <t>Covers two WEEE categories only. Denominator is waste COLLECTED, not waste generated.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="44" customHeight="1">
       <c r="A17" s="25" t="inlineStr">
         <is>
-          <t>DK.FIN.INST</t>
+          <t>DK.PAY.DIG.POS.NUM, DK.PAY.DIG.POS.VAL</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>Number of financial institutions (credit institutions) operating in Denmark.</t>
+          <t>Digital share of physical-retail payments, by NUMBER and by VALUE respectively.</t>
         </is>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>Base year 1991. Do NOT difference against DK.FIN.BRCH, which starts in 2004 - see F9_CONSOLIDATION.</t>
+          <t>Two different denominators. The value share exceeds the number share because cash survives in small transactions. Never quote one as the other, and never average them.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="44" customHeight="1">
       <c r="A18" s="25" t="inlineStr">
         <is>
-          <t>DK.FIN.EMP</t>
+          <t>DK.FIN.INST</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>Number of persons employed by Danish banks.</t>
+          <t>Number of financial institutions (credit institutions) operating in Denmark.</t>
         </is>
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>Base year 1991, so comparable with DK.FIN.INST but NOT with the branch series. Falls far less than institutions - that asymmetry is the finding in F9_CONSOLIDATION, not a data error.</t>
+          <t>Base year 1991. Do NOT difference against DK.FIN.BRCH, which starts in 2004 - see F9_CONSOLIDATION.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="44" customHeight="1">
       <c r="A19" s="25" t="inlineStr">
         <is>
+          <t>DK.FIN.EMP</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>Number of persons employed by Danish banks.</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>Base year 1991, so comparable with DK.FIN.INST but NOT with the branch series. Falls far less than institutions - that asymmetry is the finding in F9_CONSOLIDATION, not a data error.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="44" customHeight="1">
+      <c r="A20" s="25" t="inlineStr">
+        <is>
           <t>DK.SKL.1624, DK.SKL.2554, DK.SKL.5574
 (EU.SKL.1624, EU.SKL.2554, EU.SKL.5574)</t>
         </is>
       </c>
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>Individuals with at least basic overall digital skills, by age band. EU.SKL.* are the matching EU-27 comparators.</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="C20" s="15" t="inlineStr">
         <is>
           <t>Age bands, not a time series - all three are the same reference year. The DIGCOMP methodology was revised in 2021; do not join to pre-2021 skills figures.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="44" customHeight="1">
-      <c r="A20" s="25" t="inlineStr">
-        <is>
-          <t>DK.DGP.EXMP.N</t>
-        </is>
-      </c>
-      <c r="B20" s="15" t="inlineStr">
-        <is>
-          <t>Citizens formally exempt from Digital Post, as a HEADCOUNT.</t>
-        </is>
-      </c>
-      <c r="C20" s="15" t="inlineStr">
-        <is>
-          <t>A count, not a rate. Converting between this and DK.DGP.EXMP requires DK.POP.TOT and an assumption about the 15+ denominator - see 07_LIMITATIONS.</t>
         </is>
       </c>
     </row>
     <row r="21" ht="44" customHeight="1">
       <c r="A21" s="25" t="inlineStr">
         <is>
-          <t>DK.DGP.EXMP.7584, DK.DGP.EXMP.85P</t>
+          <t>DK.DGP.EXMP.N</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
         <is>
-          <t>Digital Post exemption rate within the 75-84 and 85+ age bands.</t>
+          <t>Citizens formally exempt from Digital Post, as a HEADCOUNT.</t>
         </is>
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>Denominator is the age group, not the population. These are far above the headline 4.7% and must not be compared with it directly.</t>
+          <t>A count, not a rate. Converting between this and DK.DGP.EXMP requires DK.POP.TOT and an assumption about the 15+ denominator - see 07_LIMITATIONS.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="44" customHeight="1">
       <c r="A22" s="25" t="inlineStr">
         <is>
-          <t>DK.DGX.NOUSE</t>
+          <t>DK.DGP.EXMP.7584, DK.DGP.EXMP.85P</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>Individuals who do not use digital public services at all.</t>
+          <t>Digital Post exemption rate within the 75-84 and 85+ age bands.</t>
         </is>
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>Non-use, not inability. Includes those with no need to transact as well as those unable to.</t>
+          <t>Denominator is the age group, not the population. These are far above the headline 4.7% and must not be compared with it directly.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="44" customHeight="1">
       <c r="A23" s="25" t="inlineStr">
         <is>
-          <t>DK.DGX.DISADV.LO, DK.DGX.DISADV.HI</t>
+          <t>DK.DGX.NOUSE</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>Lower and upper bound of the 'digitally disadvantaged' adult population.</t>
+          <t>Individuals who do not use digital public services at all.</t>
         </is>
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>A RANGE published as a range. Quote both bounds; citing either alone misrepresents the source's own uncertainty.</t>
+          <t>Non-use, not inability. Includes those with no need to transact as well as those unable to.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="44" customHeight="1">
       <c r="A24" s="25" t="inlineStr">
         <is>
-          <t>DK.POP.TOT</t>
+          <t>DK.DGX.DISADV.LO, DK.DGX.DISADV.HI</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>Resident population of Denmark.</t>
+          <t>Lower and upper bound of the 'digitally disadvantaged' adult population.</t>
         </is>
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>Used only as a denominator for converting headcounts to rates. Total residents, not the 15+ base the exemption rate actually uses.</t>
+          <t>A RANGE published as a range. Quote both bounds; citing either alone misrepresents the source's own uncertainty.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="44" customHeight="1">
       <c r="A25" s="25" t="inlineStr">
         <is>
-          <t>DK.TRU.DPS</t>
+          <t>DK.POP.TOT</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>Share of the population expressing trust in digital public solutions.</t>
+          <t>Resident population of Denmark.</t>
         </is>
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
-          <t>Self-reported attitude, not behaviour. High trust coexists with the exclusion measures in F4 - the two are not in contradiction.</t>
+          <t>Used only as a denominator for converting headcounts to rates. Total residents, not the 15+ base the exemption rate actually uses.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="44" customHeight="1">
       <c r="A26" s="25" t="inlineStr">
         <is>
-          <t>DK.TRU.DGP.SEC</t>
+          <t>DK.TRU.DPS</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>Share of the population perceiving Digital Post as secure.</t>
+          <t>Share of the population expressing trust in digital public solutions.</t>
         </is>
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>Narrower than DK.TRU.DPS: one service, not the whole system. Do not treat the two as one series.</t>
+          <t>Self-reported attitude, not behaviour. High trust coexists with the exclusion measures in F4 - the two are not in contradiction.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="44" customHeight="1">
       <c r="A27" s="25" t="inlineStr">
         <is>
-          <t>DK.ENT.DII</t>
+          <t>DK.TRU.DGP.SEC</t>
         </is>
       </c>
       <c r="B27" s="15" t="inlineStr">
         <is>
-          <t>SMEs reaching at least basic digital intensity (DII).</t>
+          <t>Share of the population perceiving Digital Post as secure.</t>
         </is>
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>A composite threshold count of adopted technologies, not an intensity of use. A firm clears it by adopting breadth cheaply.</t>
+          <t>Narrower than DK.TRU.DPS: one service, not the whole system. Do not treat the two as one series.</t>
         </is>
       </c>
     </row>
     <row r="28" ht="44" customHeight="1">
       <c r="A28" s="25" t="inlineStr">
         <is>
-          <t>DK.ENT.AI, DK.ENT.AI.LRG, DK.ENT.AI.SME</t>
+          <t>DK.ENT.DII</t>
         </is>
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>Enterprises adopting AI: all, large (250+) and SMEs (10-249).</t>
+          <t>SMEs reaching at least basic digital intensity (DII).</t>
         </is>
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>The headline rate is close to the SME rate because SMEs dominate by count. The large-firm gap is the real dispersion - report the split, not just the average.</t>
+          <t>A composite threshold count of adopted technologies, not an intensity of use. A firm clears it by adopting breadth cheaply.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="44" customHeight="1">
       <c r="A29" s="25" t="inlineStr">
         <is>
-          <t>DK.GOV.DPS.XB</t>
+          <t>DK.ENT.AI, DK.ENT.AI.LRG, DK.ENT.AI.SME</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
         <is>
-          <t>eGovernment Benchmark score for CROSS-BORDER citizen services.</t>
+          <t>Enterprises adopting AI: all, large (250+) and SMEs (10-249).</t>
         </is>
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>Scored against a different service basket from DK.GOV.DPS.CIT. Lower is not evidence of decline; it is a different test.</t>
+          <t>The headline rate is close to the SME rate because SMEs dominate by count. The large-firm gap is the real dispersion - report the split, not just the average.</t>
         </is>
       </c>
     </row>
     <row r="30" ht="44" customHeight="1">
       <c r="A30" s="25" t="inlineStr">
         <is>
-          <t>DK.GOV.DGP.SAVE.PLAN, DK.GOV.DGP.SAVE.VERIF</t>
+          <t>DK.GOV.DPS.XB</t>
         </is>
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>Digital Post annual public saving: as projected, and as verifiable by audit.</t>
+          <t>eGovernment Benchmark score for CROSS-BORDER citizen services.</t>
         </is>
       </c>
       <c r="C30" s="15" t="inlineStr">
         <is>
-          <t>The pair exists to be compared - the verified figure is well under half the projection. Never cite the projection alone as a realised saving.</t>
+          <t>Scored against a different service basket from DK.GOV.DPS.CIT. Lower is not evidence of decline; it is a different test.</t>
         </is>
       </c>
     </row>
     <row r="31" ht="44" customHeight="1">
       <c r="A31" s="25" t="inlineStr">
         <is>
+          <t>DK.GOV.DGP.SAVE.PLAN, DK.GOV.DGP.SAVE.VERIF</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>Digital Post annual public saving: as projected, and as verifiable by audit.</t>
+        </is>
+      </c>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>The pair exists to be compared - the verified figure is well under half the projection. Never cite the projection alone as a realised saving.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="44" customHeight="1">
+      <c r="A32" s="25" t="inlineStr">
+        <is>
           <t>DK.SME.SMVD.PROJ, DK.SME.SMVD.INV, DK.SME.SMVD.NOINV</t>
         </is>
       </c>
-      <c r="B31" s="15" t="inlineStr">
+      <c r="B32" s="15" t="inlineStr">
         <is>
           <t>SMV:Digital programme: projects supported, and participants who did or did not invest further.</t>
         </is>
       </c>
-      <c r="C31" s="15" t="inlineStr">
+      <c r="C32" s="15" t="inlineStr">
         <is>
           <t>Self-reported by participants, with no control group. Cannot support a causal claim about the programme - see the withdrawn claim in 07_LIMITATIONS and 08_AI_LOG.</t>
         </is>

</xml_diff>